<commit_message>
Updated tests with function name in descriptions
</commit_message>
<xml_diff>
--- a/Documents/Testing/Tests Documents/group5-test-cases.xlsx
+++ b/Documents/Testing/Tests Documents/group5-test-cases.xlsx
@@ -37,7 +37,23 @@
     <t>BB001</t>
   </si>
   <si>
-    <t>Verify that an engine can be added as the first car in an empty train</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[addCar()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify that an engine can be added as the first car in an empty train</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -54,7 +70,23 @@
     <t>BB002</t>
   </si>
   <si>
-    <t>Verify that a freight car can be added after an engine</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[addCar()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify that a freight car can be added after an engine</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -71,7 +103,23 @@
     <t>BB003</t>
   </si>
   <si>
-    <t>Verify engine cannot be added after freight</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[addCar()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify engine cannot be added after freight</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -89,7 +137,23 @@
     <t>BB004</t>
   </si>
   <si>
-    <t>Verify adding car exceeding MAX_WEIGHT fails</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[addCar()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify adding car exceeding MAX_WEIGHT fails</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -106,7 +170,23 @@
     <t>BB005</t>
   </si>
   <si>
-    <t>Verify removing valid car works</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[removeCar()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify removing valid car works</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -123,7 +203,23 @@
     <t>BB006</t>
   </si>
   <si>
-    <t>Verify removing invalid index fails</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[removeCar()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify removing invalid index fails</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -140,7 +236,23 @@
     <t>BB007</t>
   </si>
   <si>
-    <t>Verify removal blocked if WOOD and OIL become adjacent</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[removeCar()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify removal blocked if WOOD and OIL become adjacent</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -157,7 +269,23 @@
     <t>BB008</t>
   </si>
   <si>
-    <t>Verify last car can be removed</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[removeCar()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify last car can be removed</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -171,7 +299,23 @@
     <t>BB009</t>
   </si>
   <si>
-    <t>Verify train without engine is unsafe</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[checkTrainSafety()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify train without engine is unsafe</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -188,7 +332,23 @@
     <t>BB010</t>
   </si>
   <si>
-    <t>Verify oil after engine is unsafe</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[checkTrainSafety()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify oil after engine is unsafe</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -203,7 +363,23 @@
     <t>BB011</t>
   </si>
   <si>
-    <t>Verify WOOD next to OIL is unsafe</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[checkTrainSafety()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify WOOD next to OIL is unsafe</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -217,7 +393,23 @@
     <t>BB012</t>
   </si>
   <si>
-    <t>Verify valid configuration is safe</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[checkTrainSafety()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify valid configuration is safe</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -231,7 +423,23 @@
     <t>BB013</t>
   </si>
   <si>
-    <t>Verify displaying empty train shows message</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[displayTrain()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify displaying empty train shows message</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -247,7 +455,23 @@
     <t>BB014</t>
   </si>
   <si>
-    <t>Verify displaying one car</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[displayTrain()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify displaying one car</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -264,7 +488,23 @@
     <t>BB015</t>
   </si>
   <si>
-    <t>Verify displaying multiple cars order</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[displayTrain()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify displaying multiple cars order</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -278,7 +518,23 @@
     <t>BB016</t>
   </si>
   <si>
-    <t>Verify display handles MAX_CARS</t>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>[displayTrain()]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> Verify display handles MAX_CARS</t>
+    </r>
   </si>
   <si>
     <t>1. Initialize train
@@ -323,7 +579,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -336,6 +592,12 @@
     </font>
     <font>
       <sz val="15"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
@@ -565,9 +827,9 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -647,7 +909,7 @@
         </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -674,10 +936,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -924,9 +1186,9 @@
           <a:round/>
         </a:ln>
         <a:effectLst>
-          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
             <a:srgbClr val="000000">
-              <a:alpha val="38000"/>
+              <a:alpha val="35000"/>
             </a:srgbClr>
           </a:outerShdw>
         </a:effectLst>
@@ -1204,7 +1466,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1231,10 +1493,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">

</xml_diff>